<commit_message>
feat: migrate admin frontend to React (Vite) and unify GeneratePersona layout
- Scaffold React + Vite frontend with component-based architecture
- Add Sidebar, GeneratePersona, CrewProcess, ExecutionHistory,
  NodeFlowDesigner, McpCatalog components
- Consolidate GeneratePersona into a single-frame layout with title
  at the top instead of 2-column aside/main split
- Update Dockerfile and app.py to serve the new frontend
- Update persona_generate spec and generate.py
</commit_message>
<xml_diff>
--- a/dev/company-crew-dev/crew_specs/persona_generate.xlsx
+++ b/dev/company-crew-dev/crew_specs/persona_generate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jck/WORK/DEV/company-crewai-amp-v2/dev/company-crew-dev/crew_specs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5FCFE78-81AE-A74B-A3BF-0E298DC1EBA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3162865-D6D0-DF4E-AE45-DB15231B8DB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{1B6F41E7-F757-EF41-AEAE-051A461303B9}"/>
   </bookViews>
@@ -305,24 +305,25 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">입력 받은 업무 목적 (business_goal) {business_goal} , 단계별 tool 유형 (step_tools) {step_tools} 을 기준으로  crewai agent 에서 필요한 config jsonc (task.jsonc, agent.jsonc) 을 만들기 위한 spec 파일을 생성한다.  
-Step_tools 은  step:tool 의 json 형태로 구성되고 tool 은 없을 수도 있으며 mcp_tool 과 연결된다. 
+    <t>사용자가 입력한 business_goal, step_tools 을 잘 이해하고 crewai agent 가 만들어질 수 있도록 각 세부 속성을 자동으로 만들어야 한다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>crewai 프레임워크, sdk 를 잘 이해하고 sdk 기반으로 실제 agent 를 작성한 경험이 풍부하다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>task_name,  task_context, task_description, task_expected_output, task_output_file, task_agent, agent_role, agent_goal, agent_backstory, agent_tools 을  markdown 표 형태로  출력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">입력 받은 업무 목적 (business_goal) "{business_goal}" , 단계별 tool 유형 (step_tools) "{step_tools}" 을 기준으로  crewai agent 에서 필요한 config jsonc (task.jsonc, agent.jsonc) 을 만들기 위한 spec 파일을 생성한다.  
+Step_tools 은  step:tool 의 리스트 형태로 구성되고 tool 은 mcp_tool 과 연결되며, 없을 수도 있다. 
 Spec 파일의 행은 step 별로 작성되어야 한다. 
 각 step 의 명칭과 업무목적을 조합해서 task_name 을 명명한다. 
+각 step 과 도구를 조합해서  mcp tool list 를 조회하여 연관된 tool 을 agent_tools 로 설정한다. 
 그외 task, agent 에서 필요한 속성은  각각 task_xxxx,  agent_xxxx 형태로 정의하고,  해당 내용은 crewai sdk 에서 인식될 수 있도록  자동으로 작성한다.
 </t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>사용자가 입력한 business_goal, step_tools 을 잘 이해하고 crewai agent 가 만들어질 수 있도록 각 세부 속성을 자동으로 만들어야 한다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>crewai 프레임워크, sdk 를 잘 이해하고 sdk 기반으로 실제 agent 를 작성한 경험이 풍부하다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>task_name,  task_context, task_description, task_expected_output, task_output_file, task_agent, agent_role, agent_goal, agent_backstory, agent_tools 을  markdown 표 형태로  출력</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -905,10 +906,10 @@
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>48</v>
@@ -920,10 +921,10 @@
         <v>50</v>
       </c>
       <c r="H2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>53</v>
       </c>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>

</xml_diff>

<commit_message>
Fix generate.sh syntax and add work_type to persona_generate spec
- generate.sh: add missing `then` to the if statement, use `-z` with a
  quoted variable to check for an empty argument, quote the crew_name
  argument, add a bash shebang, and exit 1 on usage error
- persona_generate.xlsx: add the work_type ({work_type}) input to the
  generate_persona task description
</commit_message>
<xml_diff>
--- a/dev/company-crew-dev/crew_specs/persona_generate.xlsx
+++ b/dev/company-crew-dev/crew_specs/persona_generate.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jck/WORK/DEV/company-crewai-amp-v2/dev/company-crew-dev/crew_specs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3E2B4EC-6FF6-6B4F-A95B-8078E54B62B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1373E19-0217-D247-89D3-FCFE0C5B2775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{1B6F41E7-F757-EF41-AEAE-051A461303B9}"/>
   </bookViews>
@@ -309,11 +309,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>사용자가 입력한 persona_name, business_goal, step_tools 을 잘 이해하고 crewai agent 가 만들어질 수 있도록 각 세부 속성을 자동으로 만들어야 한다. 
-Crew spec 문서는 한글로 만들어야 한다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>all.mcp.list</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -322,21 +317,26 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>입력 받은 페르소나 이름 (persona_name) "{persona_name}", 업무 유형 (work_type) "{work_type}", 업무 목적 (business_goal) "{business_goal}" , 단계별 tool 유형 (step_tools) "{step_tools}" 을 기준으로  crewai agent 에서 필요한 config jsonc (task.jsonc, agent.jsonc) 을 만들기 위한 spec 파일을 생성한다.  spec 파일은  step 별로 task 로 매칭되어 각 행라인으로 작성한다.
-step_tools 은  step:tool_list 의 리스트 형태로 구성되고 각각의 tool 은 mcp와 연결되며, 연결된 tool 은 없을 수도 있다. 아래 예시를 참조해줘.
+    <t>입력 받은 페르소나 이름 (persona_name) "{persona_name}", 업무 유형 (work_type) "{work_type}", 업무 목적 (business_goal) "{business_goal}" , 단계별 tool 유형 (step_tools) "{step_tools}" 을 기준으로  crewai agent 에서 필요한 config jsonc (task.jsonc, agent.jsonc) 을 만들기 위한 spec 파일을 생성합니다.  spec 파일은  step 별로 task 로 매칭되어 각 행라인으로 작성합니다.
+step_tools 은  step:tool_list 의 리스트 형태로 구성되고 각각의 tool 은 mcp와 연결되며, 연결된 tool 은 없을 수도 있습니다. 아래 예시를 참조해주세요.
   "step_tools": [
     "extract:[database,datadog]",
     "analysis",
     "report"
   ]  
-위 work_type,  business_goal 정보를 토대로 crewai config 속성을 작성해줘
+위 work_type,  business_goal 정보를 토대로 crewai config 속성을 작성해주세요.
 . crew_name :  persona_name 을 영어로 번역하여 설정 (output_file markdown 문서의 이름)
 . task_name : 각 step 의 명칭과 업무목적을 조합해서 단위 프로세스를 명명 (반드시 영어로 작성) 
 . task_context : 이전 step 과 연결될 경우 이전 task_name 을 그대로 작성
 . task_agent : 각 step 의 명칭과 업무목적을 조합해서 수행하는 역할자 설정 (반드시 영어로 작성)
 . mcp : step 과 tool명 을 조합하고 all.mcp.list tool 에서 mcp_name (response.tools.name)을 가져와서 매칭   
-. 그외 task, agent 에서 필요한 속성은  각각 task_xxxx,  agent_xxxx 형태로 정의하고,  해당 내용은 crewai sdk 에서 인식될 수 있도록  자동으로 작성한다. (한글로 작성) 
-. crew_name 은 변수로 저장하여 output_file 의 명칭으로 사용한다.</t>
+. 그외 task, agent 에서 필요한 속성은  각각 task_xxxx,  agent_xxxx 형태로 정의하고,  해당 내용은 crewai sdk 에서 인식될 수 있도록  자동으로 작성해주세요. (한글로 작성) 
+. crew_name 은 변수로 저장하여 output_file 의 명칭으로 사용합니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>사용자가 입력한 persona_name, business_goal, work_type, step_tools 을 잘 이해하고 crewai agent 가 만들어질 수 있도록 각 세부 속성을 자동으로 만들어야 한다. 
+Crew spec 문서는 한글로 만들어야 한다.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -919,13 +919,13 @@
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>51</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>48</v>
@@ -934,13 +934,13 @@
         <v>50</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>49</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K2" s="4"/>
     </row>

</xml_diff>